<commit_message>
first commit - commiting changes to release branch
</commit_message>
<xml_diff>
--- a/alfred_requirements.xlsx
+++ b/alfred_requirements.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="354">
   <si>
     <t xml:space="preserve">req_id</t>
   </si>
@@ -1094,6 +1094,9 @@
   </si>
   <si>
     <t xml:space="preserve">xxx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yyy</t>
   </si>
   <si>
     <t xml:space="preserve">REQ04_BAT01_TC03</t>
@@ -1562,7 +1565,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C28"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="43.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="155.86"/>
@@ -1860,9 +1863,9 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E64"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="82"/>
@@ -2764,7 +2767,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="91.15"/>
@@ -2957,7 +2960,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C76"/>
-  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="255.71"/>
   </cols>
@@ -3636,7 +3639,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Z26"/>
-  <sheetFormatPr defaultColWidth="9.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.14"/>
@@ -3819,52 +3822,57 @@
         <v>336</v>
       </c>
     </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>337</v>
+      </c>
+    </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q11" s="34"/>
       <c r="R11" s="34"/>
       <c r="S11" s="34"/>
       <c r="T11" s="34"/>
       <c r="U11" s="20" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="V11" s="20" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="W11" s="20" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="X11" s="20"/>
       <c r="Y11" s="20"/>
       <c r="Z11" s="35" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q12" s="8" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="R12" s="8" t="s">
         <v>60</v>
       </c>
       <c r="S12" s="8" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="T12" s="8" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="U12" s="20" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="V12" s="20" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="W12" s="20" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="X12" s="20"/>
       <c r="Y12" s="20"/>
       <c r="Z12" s="35" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3873,23 +3881,23 @@
       <c r="S13" s="8"/>
       <c r="T13" s="8"/>
       <c r="U13" s="20" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="V13" s="20" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="W13" s="20" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="X13" s="20"/>
       <c r="Y13" s="20"/>
       <c r="Z13" s="35" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="36" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B15" s="36"/>
       <c r="C15" s="36"/>
@@ -3921,13 +3929,13 @@
       <c r="G16" s="37"/>
       <c r="H16" s="37"/>
       <c r="I16" s="5" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="K16" s="37" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
first commit - dev branch
</commit_message>
<xml_diff>
--- a/alfred_requirements.xlsx
+++ b/alfred_requirements.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="355">
   <si>
     <t xml:space="preserve">req_id</t>
   </si>
@@ -1097,6 +1097,9 @@
   </si>
   <si>
     <t xml:space="preserve">yyy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zzz</t>
   </si>
   <si>
     <t xml:space="preserve">REQ04_BAT01_TC03</t>
@@ -3639,7 +3642,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Z26"/>
-  <sheetFormatPr defaultColWidth="9.16015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.14"/>
@@ -3828,51 +3831,54 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>338</v>
+      </c>
       <c r="Q11" s="34"/>
       <c r="R11" s="34"/>
       <c r="S11" s="34"/>
       <c r="T11" s="34"/>
       <c r="U11" s="20" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="V11" s="20" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="W11" s="20" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="X11" s="20"/>
       <c r="Y11" s="20"/>
       <c r="Z11" s="35" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="Q12" s="8" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="R12" s="8" t="s">
         <v>60</v>
       </c>
       <c r="S12" s="8" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="T12" s="8" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="U12" s="20" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="V12" s="20" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="W12" s="20" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="X12" s="20"/>
       <c r="Y12" s="20"/>
       <c r="Z12" s="35" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3881,23 +3887,23 @@
       <c r="S13" s="8"/>
       <c r="T13" s="8"/>
       <c r="U13" s="20" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="V13" s="20" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="W13" s="20" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="X13" s="20"/>
       <c r="Y13" s="20"/>
       <c r="Z13" s="35" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="36" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B15" s="36"/>
       <c r="C15" s="36"/>
@@ -3929,13 +3935,13 @@
       <c r="G16" s="37"/>
       <c r="H16" s="37"/>
       <c r="I16" s="5" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="K16" s="37" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
added abracadabra to main
</commit_message>
<xml_diff>
--- a/alfred_requirements.xlsx
+++ b/alfred_requirements.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="355">
   <si>
     <t xml:space="preserve">req_id</t>
   </si>
@@ -1106,6 +1106,9 @@
   </si>
   <si>
     <t xml:space="preserve">Validate error pop-ups at different soc thresholds, i.e. 19% , 9% , 5% , 2%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abracadabra</t>
   </si>
   <si>
     <t xml:space="preserve">REQ04_BAT02</t>
@@ -3639,7 +3642,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Z26"/>
-  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.171875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13.71"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.14"/>
@@ -3848,31 +3851,34 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="0" t="s">
+        <v>341</v>
+      </c>
       <c r="Q12" s="8" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="R12" s="8" t="s">
         <v>60</v>
       </c>
       <c r="S12" s="8" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="T12" s="8" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="U12" s="20" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="V12" s="20" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="W12" s="20" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="X12" s="20"/>
       <c r="Y12" s="20"/>
       <c r="Z12" s="35" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3881,23 +3887,23 @@
       <c r="S13" s="8"/>
       <c r="T13" s="8"/>
       <c r="U13" s="20" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="V13" s="20" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="W13" s="20" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="X13" s="20"/>
       <c r="Y13" s="20"/>
       <c r="Z13" s="35" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="36" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B15" s="36"/>
       <c r="C15" s="36"/>
@@ -3929,13 +3935,13 @@
       <c r="G16" s="37"/>
       <c r="H16" s="37"/>
       <c r="I16" s="5" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="K16" s="37" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>